<commit_message>
Added Shielded RJ connector w/ LEDs
</commit_message>
<xml_diff>
--- a/To Add v2/Connectors - RJ.xlsx
+++ b/To Add v2/Connectors - RJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\To Add v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5119B957-D0AF-4C03-8D4A-CDAAE541ED85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7AC0F3C-410D-4CB6-BD79-EA4B3D58877B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39960" yWindow="10590" windowWidth="19200" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
-  <si>
-    <t>Remember to modify the Kicad DBL!!!</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="52">
   <si>
     <t>Remember to add to the database!!!</t>
   </si>
@@ -177,6 +174,24 @@
   </si>
   <si>
     <t>Connectors:MTJ-661X1</t>
+  </si>
+  <si>
+    <t>2057-MTJ-88ARX1-FSM-LG-ND</t>
+  </si>
+  <si>
+    <t>MTJ-88ARX1-FSM-LG</t>
+  </si>
+  <si>
+    <t>Shielded, LEDs</t>
+  </si>
+  <si>
+    <t>https://app.adam-tech.com/products/download/data_sheet/203879/mtj-88arx1-fsm-lg-data-sheet.pdf</t>
+  </si>
+  <si>
+    <t>0Dan_Connectors:8P8C_LED_Shielded_x2_GY</t>
+  </si>
+  <si>
+    <t>Connectors:ADAMTECH_MTJ-88ARX1-FSM-LG</t>
   </si>
 </sst>
 </file>
@@ -226,7 +241,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -503,226 +526,224 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="B1" s="1"/>
+      <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:Q2" si="0">COUNTA(C7:C9999)</f>
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="J2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="O2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="Q2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="X2" t="s">
         <v>2</v>
-      </c>
-      <c r="C2">
-        <f>COUNTA(C7:C9999)</f>
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <f>COUNTA(D7:D9999)</f>
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <f>COUNTA(E7:E9999)</f>
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <f>COUNTA(F7:F9999)</f>
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <f>COUNTA(G7:G9999)</f>
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <f>COUNTA(H7:H9999)</f>
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <f>COUNTA(I7:I9999)</f>
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <f>COUNTA(J7:J9999)</f>
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <f>COUNTA(K7:K9999)</f>
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <f>COUNTA(L7:L9999)</f>
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <f>COUNTA(M7:M9999)</f>
-        <v>2</v>
-      </c>
-      <c r="N2">
-        <f>COUNTA(N7:N9999)</f>
-        <v>2</v>
-      </c>
-      <c r="O2">
-        <f>COUNTA(O7:O9999)</f>
-        <v>2</v>
-      </c>
-      <c r="P2">
-        <f>COUNTA(P7:P9999)</f>
-        <v>2</v>
-      </c>
-      <c r="Q2">
-        <f>COUNTA(Q7:Q9999)</f>
-        <v>2</v>
-      </c>
-      <c r="X2" t="s">
-        <v>3</v>
       </c>
       <c r="Y2">
         <f>AVERAGE(U7:U9999)</f>
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="X3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Y3">
         <f>MAX(C2:Q2)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="X4" t="s">
         <v>5</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-      <c r="N4">
-        <v>1</v>
-      </c>
-      <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="P4">
-        <v>1</v>
-      </c>
-      <c r="Q4">
-        <v>1</v>
-      </c>
-      <c r="X4" t="s">
-        <v>6</v>
       </c>
       <c r="Y4">
         <f>SUM(V7:V9999)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="X5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y5">
         <f>COUNTIF(U7:U9999,"&lt;100")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>10</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>11</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>12</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>13</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>14</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>15</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="T6" t="s">
         <v>17</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>18</v>
       </c>
-      <c r="U6" t="s">
+      <c r="V6" t="s">
         <v>19</v>
       </c>
-      <c r="V6" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -735,43 +756,43 @@
         <v>RJ45 R/A</v>
       </c>
       <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>29</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>30</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>31</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>32</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>33</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>34</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>35</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>36</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>37</v>
       </c>
-      <c r="P7" t="s">
-        <v>38</v>
-      </c>
       <c r="Q7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T7">
         <f>COUNTBLANK(C7:Q7)</f>
@@ -786,14 +807,14 @@
         <v>1</v>
       </c>
       <c r="X7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="Y7">
         <f>SUM(C4:Q4)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2</v>
       </c>
@@ -806,43 +827,43 @@
         <v>RJ25 R/A</v>
       </c>
       <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" t="s">
+        <v>30</v>
+      </c>
+      <c r="J8" t="s">
         <v>40</v>
       </c>
-      <c r="G8" t="s">
-        <v>29</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="K8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" t="s">
+        <v>42</v>
+      </c>
+      <c r="N8" t="s">
+        <v>43</v>
+      </c>
+      <c r="O8" t="s">
+        <v>44</v>
+      </c>
+      <c r="P8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q8" t="s">
         <v>30</v>
-      </c>
-      <c r="I8" t="s">
-        <v>31</v>
-      </c>
-      <c r="J8" t="s">
-        <v>41</v>
-      </c>
-      <c r="K8" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M8" t="s">
-        <v>43</v>
-      </c>
-      <c r="N8" t="s">
-        <v>44</v>
-      </c>
-      <c r="O8" t="s">
-        <v>45</v>
-      </c>
-      <c r="P8" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>31</v>
       </c>
       <c r="T8">
         <f>COUNTBLANK(C8:Q8)</f>
@@ -857,21 +878,68 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="C9" t="str">
+        <f>_xlfn.CONCAT(F9," ",D9," ",G9," ",I9," ",Q9)</f>
+        <v>8P8C RJ45 R/A Through Hole Shielded, LEDs  </v>
+      </c>
+      <c r="D9" t="str">
+        <f>_xlfn.CONCAT(E9," ",H9)</f>
+        <v>RJ45 R/A</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K9" t="s">
+        <v>47</v>
+      </c>
+      <c r="L9" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" t="s">
+        <v>46</v>
+      </c>
+      <c r="N9" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" t="s">
+        <v>50</v>
+      </c>
+      <c r="P9" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>30</v>
+      </c>
       <c r="T9">
         <f>COUNTBLANK(C9:Q9)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="U9">
         <f>100*COUNTA(C9:Q9)/$Y$7</f>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V9">
-        <f t="shared" ref="V9:V10" si="0">IF(U9=100,1,0)</f>
-        <v>0</v>
+        <f t="shared" ref="V9:V10" si="1">IF(U9=100,1,0)</f>
+        <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="T10">
         <f>COUNTBLANK(C10:Q10)</f>
         <v>15</v>
@@ -881,11 +949,16 @@
         <v>0</v>
       </c>
       <c r="V10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C7:Q53">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(C7))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>